<commit_message>
BugFix ArrowPosition getting stuck
</commit_message>
<xml_diff>
--- a/Diagramme/SmartClock_Gantt-Diagramm_V2.xlsx
+++ b/Diagramme/SmartClock_Gantt-Diagramm_V2.xlsx
@@ -1,7 +1,7 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
   <workbookPr filterPrivacy="1" codeName="ThisWorkbook"/>
   <xr:revisionPtr revIDLastSave="697" documentId="8_{0C4EAEB1-A5C4-4402-980F-B32D81185735}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{64EE4A6D-F461-4C5D-B572-20DCEA631B00}"/>
   <bookViews>
@@ -259,7 +259,7 @@
     <numFmt numFmtId="165" formatCode="d"/>
     <numFmt numFmtId="166" formatCode="#,##0_ ;\-#,##0\ "/>
   </numFmts>
-  <fonts count="36" x14ac:knownFonts="1">
+  <fonts count="36">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1169,6 +1169,33 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="13" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="9" borderId="0" xfId="5" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="5" borderId="0" xfId="11" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="32" fillId="13" borderId="0" xfId="6" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -1187,34 +1214,7 @@
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="5" borderId="0" xfId="11" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="9" borderId="0" xfId="5" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="25" fillId="13" borderId="0" xfId="5" applyFont="1" applyFill="1" applyAlignment="1">
@@ -1693,36 +1693,6 @@
       </fill>
     </dxf>
     <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="1" relativeIndent="1" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <strike val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="12"/>
-        <color auto="1"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor theme="0" tint="-0.14999847407452621"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
       <font>
         <strike val="0"/>
         <outline val="0"/>
@@ -1834,6 +1804,36 @@
         <patternFill patternType="solid">
           <fgColor indexed="64"/>
           <bgColor theme="1" tint="0.249977111117893"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="1" relativeIndent="1" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <color auto="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor theme="0" tint="-0.14999847407452621"/>
         </patternFill>
       </fill>
     </dxf>
@@ -2174,7 +2174,7 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{DD82988E-1813-40AE-BDE7-9F0200A703CB}" name="Meilensteine4352" displayName="Meilensteine4352" ref="B9:G36" totalsRowShown="0" headerRowDxfId="42" dataDxfId="41">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{DD82988E-1813-40AE-BDE7-9F0200A703CB}" name="Meilensteine4352" displayName="Meilensteine4352" ref="B9:G36" totalsRowShown="0" headerRowDxfId="38" dataDxfId="37">
   <autoFilter ref="B9:G36" xr:uid="{29E5A880-80D5-4B65-B5FB-8FB3913D3D27}">
     <filterColumn colId="0" hiddenButton="1"/>
     <filterColumn colId="1" hiddenButton="1"/>
@@ -2184,12 +2184,12 @@
     <filterColumn colId="5" hiddenButton="1"/>
   </autoFilter>
   <tableColumns count="6">
-    <tableColumn id="1" xr3:uid="{619BF8F6-D0F1-41AD-871D-FE0240C45A93}" name="Meilensteinbeschreibung" dataDxfId="40"/>
-    <tableColumn id="2" xr3:uid="{39BD914E-FB02-4352-846C-6D59624DC0B0}" name="Kategorie" dataDxfId="39"/>
-    <tableColumn id="3" xr3:uid="{D274194F-BCA0-44F3-84B2-217254EE241C}" name="Zeitaufwand in std" dataDxfId="38"/>
-    <tableColumn id="4" xr3:uid="{8385BC6F-56EE-4363-A106-8DB0A1E4EF5A}" name="Fortschritt" dataDxfId="37"/>
-    <tableColumn id="5" xr3:uid="{02926609-7B93-4B6F-BE96-92EC7A949E4B}" name="Start" dataDxfId="36" dataCellStyle="Datum"/>
-    <tableColumn id="6" xr3:uid="{8FF9BE8E-04B7-4B39-AC27-D2E534204BC3}" name="Tage" dataDxfId="35"/>
+    <tableColumn id="1" xr3:uid="{619BF8F6-D0F1-41AD-871D-FE0240C45A93}" name="Meilensteinbeschreibung" dataDxfId="36"/>
+    <tableColumn id="2" xr3:uid="{39BD914E-FB02-4352-846C-6D59624DC0B0}" name="Kategorie" dataDxfId="35"/>
+    <tableColumn id="3" xr3:uid="{D274194F-BCA0-44F3-84B2-217254EE241C}" name="Zeitaufwand in std" dataDxfId="34"/>
+    <tableColumn id="4" xr3:uid="{8385BC6F-56EE-4363-A106-8DB0A1E4EF5A}" name="Fortschritt" dataDxfId="33"/>
+    <tableColumn id="5" xr3:uid="{02926609-7B93-4B6F-BE96-92EC7A949E4B}" name="Start" dataDxfId="32" dataCellStyle="Datum"/>
+    <tableColumn id="6" xr3:uid="{8FF9BE8E-04B7-4B39-AC27-D2E534204BC3}" name="Tage" dataDxfId="31"/>
   </tableColumns>
   <tableStyleInfo name="Aufgabenliste" showFirstColumn="1" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
   <extLst>
@@ -2201,7 +2201,7 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{0EDB95CA-98FE-4198-8801-690B9B480FDF}" name="Meilensteine435" displayName="Meilensteine435" ref="B9:G36" totalsRowShown="0" headerRowDxfId="34">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{0EDB95CA-98FE-4198-8801-690B9B480FDF}" name="Meilensteine435" displayName="Meilensteine435" ref="B9:G36" totalsRowShown="0" headerRowDxfId="42">
   <autoFilter ref="B9:G36" xr:uid="{29E5A880-80D5-4B65-B5FB-8FB3913D3D27}">
     <filterColumn colId="0" hiddenButton="1"/>
     <filterColumn colId="1" hiddenButton="1"/>
@@ -2211,9 +2211,9 @@
     <filterColumn colId="5" hiddenButton="1"/>
   </autoFilter>
   <tableColumns count="6">
-    <tableColumn id="1" xr3:uid="{6E47A83D-ACD7-4EB6-9B84-5195E813945E}" name="Meilensteinbeschreibung" dataDxfId="33"/>
-    <tableColumn id="2" xr3:uid="{529EEF64-D037-4ACF-8CA4-0C10FE2D1FBB}" name="Kategorie" dataDxfId="32"/>
-    <tableColumn id="3" xr3:uid="{711D01BA-2785-403A-9636-CCC7E2ADA584}" name="Aufwand Soll / Ist" dataDxfId="31"/>
+    <tableColumn id="1" xr3:uid="{6E47A83D-ACD7-4EB6-9B84-5195E813945E}" name="Meilensteinbeschreibung" dataDxfId="41"/>
+    <tableColumn id="2" xr3:uid="{529EEF64-D037-4ACF-8CA4-0C10FE2D1FBB}" name="Kategorie" dataDxfId="40"/>
+    <tableColumn id="3" xr3:uid="{711D01BA-2785-403A-9636-CCC7E2ADA584}" name="Aufwand Soll / Ist" dataDxfId="39"/>
     <tableColumn id="4" xr3:uid="{62B00BEF-16BE-4692-B5E2-F287F680F2C1}" name="Fortschritt"/>
     <tableColumn id="5" xr3:uid="{D6D72902-F68F-4E59-A714-AFFF520C647A}" name="Start" dataCellStyle="Datum"/>
     <tableColumn id="6" xr3:uid="{93E698DE-286F-49ED-AA20-D0C843671DE8}" name="Tage"/>
@@ -2519,7 +2519,7 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <sheetPr codeName="Sheet2"/>
   <dimension ref="A1:M19"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="12.75"/>
   <cols>
     <col min="1" max="1" width="4.7109375" style="8" customWidth="1"/>
     <col min="2" max="2" width="2.7109375" style="8" customWidth="1"/>
@@ -2528,17 +2528,17 @@
     <col min="7" max="16384" width="9.140625" style="6"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" s="7" customFormat="1" ht="28.5" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:13" s="7" customFormat="1" ht="28.5">
       <c r="D1" s="104"/>
     </row>
-    <row r="2" spans="1:13" ht="50.1" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:13" ht="50.1" customHeight="1">
       <c r="A2" s="7"/>
       <c r="B2" s="110"/>
-      <c r="C2" s="124" t="s">
+      <c r="C2" s="133" t="s">
         <v>0</v>
       </c>
-      <c r="D2" s="124"/>
-      <c r="E2" s="124"/>
+      <c r="D2" s="133"/>
+      <c r="E2" s="133"/>
       <c r="F2" s="110"/>
       <c r="G2" s="7"/>
       <c r="H2" s="7"/>
@@ -2548,7 +2548,7 @@
       <c r="L2" s="7"/>
       <c r="M2" s="7"/>
     </row>
-    <row r="3" spans="1:13" ht="14.45" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:13" ht="14.45" customHeight="1">
       <c r="A3" s="7"/>
       <c r="B3" s="105"/>
       <c r="C3" s="106"/>
@@ -2563,14 +2563,14 @@
       <c r="L3" s="7"/>
       <c r="M3" s="7"/>
     </row>
-    <row r="4" spans="1:13" s="8" customFormat="1" ht="75" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:13" s="8" customFormat="1" ht="75" customHeight="1">
       <c r="A4" s="7"/>
       <c r="B4" s="105"/>
-      <c r="C4" s="125" t="s">
+      <c r="C4" s="134" t="s">
         <v>1</v>
       </c>
-      <c r="D4" s="125"/>
-      <c r="E4" s="125"/>
+      <c r="D4" s="134"/>
+      <c r="E4" s="134"/>
       <c r="F4" s="105"/>
       <c r="G4" s="7"/>
       <c r="H4" s="7"/>
@@ -2580,14 +2580,14 @@
       <c r="L4" s="7"/>
       <c r="M4" s="7"/>
     </row>
-    <row r="5" spans="1:13" s="8" customFormat="1" ht="75" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:13" s="8" customFormat="1" ht="75" customHeight="1">
       <c r="A5" s="7"/>
       <c r="B5" s="105"/>
-      <c r="C5" s="125" t="s">
+      <c r="C5" s="134" t="s">
         <v>2</v>
       </c>
-      <c r="D5" s="125"/>
-      <c r="E5" s="125"/>
+      <c r="D5" s="134"/>
+      <c r="E5" s="134"/>
       <c r="F5" s="105"/>
       <c r="G5" s="7"/>
       <c r="H5" s="7"/>
@@ -2597,7 +2597,7 @@
       <c r="L5" s="7"/>
       <c r="M5" s="7"/>
     </row>
-    <row r="6" spans="1:13" ht="15" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:13" ht="15">
       <c r="A6" s="6"/>
       <c r="B6" s="108"/>
       <c r="C6" s="108"/>
@@ -2605,15 +2605,15 @@
       <c r="E6" s="108"/>
       <c r="F6" s="108"/>
     </row>
-    <row r="7" spans="1:13" ht="50.1" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:13" ht="50.1" customHeight="1">
       <c r="A7" s="6"/>
       <c r="B7" s="6"/>
     </row>
-    <row r="8" spans="1:13" ht="14.45" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:13" ht="14.45" customHeight="1">
       <c r="A8" s="6"/>
       <c r="B8" s="6"/>
     </row>
-    <row r="9" spans="1:13" ht="90" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:13" ht="90" customHeight="1">
       <c r="C9" s="8"/>
       <c r="D9" s="8"/>
       <c r="E9" s="8"/>
@@ -2621,51 +2621,51 @@
       <c r="G9" s="8"/>
       <c r="H9" s="8"/>
     </row>
-    <row r="10" spans="1:13" ht="14.45" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:13" ht="14.45" customHeight="1">
       <c r="A10" s="6"/>
       <c r="B10" s="6"/>
     </row>
-    <row r="11" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:13">
       <c r="A11" s="6"/>
       <c r="B11" s="6"/>
       <c r="D11" s="8"/>
     </row>
-    <row r="12" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:13">
       <c r="A12" s="6"/>
       <c r="B12" s="6"/>
       <c r="D12" s="8"/>
     </row>
-    <row r="13" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:13">
       <c r="A13" s="6"/>
       <c r="B13" s="6"/>
       <c r="D13" s="8"/>
     </row>
-    <row r="14" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:13">
       <c r="A14" s="6"/>
       <c r="B14" s="6"/>
       <c r="D14" s="8"/>
     </row>
-    <row r="15" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:13">
       <c r="A15" s="6"/>
       <c r="B15" s="6"/>
       <c r="D15" s="8"/>
     </row>
-    <row r="16" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:13">
       <c r="A16" s="6"/>
       <c r="B16" s="6"/>
       <c r="D16" s="8"/>
     </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:4">
       <c r="A17" s="6"/>
       <c r="B17" s="6"/>
       <c r="D17" s="8"/>
     </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:4">
       <c r="A18" s="6"/>
       <c r="B18" s="6"/>
       <c r="D18" s="8"/>
     </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:4">
       <c r="A19" s="6"/>
       <c r="B19" s="6"/>
       <c r="D19" s="8"/>
@@ -2688,7 +2688,7 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:BP38"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="30" customHeight="1" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="30" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="4.7109375" style="9" customWidth="1"/>
     <col min="2" max="2" width="37.85546875" customWidth="1"/>
@@ -2702,30 +2702,30 @@
     <col min="65" max="65" width="2.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:68" ht="25.15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="2" spans="1:68" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:68" ht="25.15" customHeight="1"/>
+    <row r="2" spans="1:68" ht="49.9" customHeight="1">
       <c r="A2" s="10"/>
-      <c r="B2" s="127" t="s">
+      <c r="B2" s="136" t="s">
         <v>39</v>
       </c>
-      <c r="C2" s="127"/>
-      <c r="D2" s="127"/>
-      <c r="E2" s="127"/>
-      <c r="F2" s="127"/>
-      <c r="G2" s="127"/>
-      <c r="H2" s="127"/>
-      <c r="I2" s="128"/>
-      <c r="J2" s="128"/>
-      <c r="K2" s="128"/>
-      <c r="L2" s="128"/>
-      <c r="M2" s="128"/>
-      <c r="N2" s="128"/>
-      <c r="O2" s="129"/>
-      <c r="P2" s="129"/>
-      <c r="Q2" s="129"/>
-      <c r="R2" s="129"/>
-      <c r="S2" s="129"/>
-      <c r="T2" s="129"/>
+      <c r="C2" s="136"/>
+      <c r="D2" s="136"/>
+      <c r="E2" s="136"/>
+      <c r="F2" s="136"/>
+      <c r="G2" s="136"/>
+      <c r="H2" s="136"/>
+      <c r="I2" s="137"/>
+      <c r="J2" s="137"/>
+      <c r="K2" s="137"/>
+      <c r="L2" s="137"/>
+      <c r="M2" s="137"/>
+      <c r="N2" s="137"/>
+      <c r="O2" s="138"/>
+      <c r="P2" s="138"/>
+      <c r="Q2" s="138"/>
+      <c r="R2" s="138"/>
+      <c r="S2" s="138"/>
+      <c r="T2" s="138"/>
       <c r="U2" s="64"/>
       <c r="V2" s="64"/>
       <c r="W2" s="64"/>
@@ -2772,7 +2772,7 @@
       <c r="BL2" s="64"/>
       <c r="BM2" s="64"/>
     </row>
-    <row r="3" spans="1:68" ht="19.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:68" ht="19.899999999999999" customHeight="1">
       <c r="A3" s="10"/>
       <c r="B3" s="65"/>
       <c r="C3" s="66"/>
@@ -2786,7 +2786,7 @@
       <c r="K3" s="1"/>
       <c r="L3" s="1"/>
     </row>
-    <row r="4" spans="1:68" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:68" ht="30" customHeight="1">
       <c r="A4" s="10"/>
       <c r="B4" s="69" t="s">
         <v>36</v>
@@ -2799,40 +2799,40 @@
         <v>30</v>
       </c>
       <c r="H4" s="72"/>
-      <c r="I4" s="130" t="s">
+      <c r="I4" s="129" t="s">
         <v>25</v>
       </c>
-      <c r="J4" s="130"/>
-      <c r="K4" s="130"/>
-      <c r="L4" s="130"/>
-      <c r="M4" s="130"/>
-      <c r="N4" s="130"/>
-      <c r="P4" s="131"/>
-      <c r="Q4" s="131"/>
-      <c r="R4" s="131"/>
-      <c r="S4" s="131"/>
-      <c r="T4" s="131"/>
-      <c r="U4" s="131"/>
-      <c r="W4" s="131"/>
-      <c r="X4" s="131"/>
-      <c r="Y4" s="131"/>
-      <c r="Z4" s="131"/>
-      <c r="AA4" s="131"/>
-      <c r="AB4" s="131"/>
-      <c r="AD4" s="131"/>
-      <c r="AE4" s="131"/>
-      <c r="AF4" s="131"/>
-      <c r="AG4" s="131"/>
-      <c r="AH4" s="131"/>
-      <c r="AJ4" s="126"/>
-      <c r="AK4" s="126"/>
-      <c r="AL4" s="126"/>
-      <c r="AM4" s="126"/>
-      <c r="AN4" s="126"/>
-      <c r="AO4" s="126"/>
-      <c r="AP4" s="126"/>
+      <c r="J4" s="129"/>
+      <c r="K4" s="129"/>
+      <c r="L4" s="129"/>
+      <c r="M4" s="129"/>
+      <c r="N4" s="129"/>
+      <c r="P4" s="139"/>
+      <c r="Q4" s="139"/>
+      <c r="R4" s="139"/>
+      <c r="S4" s="139"/>
+      <c r="T4" s="139"/>
+      <c r="U4" s="139"/>
+      <c r="W4" s="139"/>
+      <c r="X4" s="139"/>
+      <c r="Y4" s="139"/>
+      <c r="Z4" s="139"/>
+      <c r="AA4" s="139"/>
+      <c r="AB4" s="139"/>
+      <c r="AD4" s="139"/>
+      <c r="AE4" s="139"/>
+      <c r="AF4" s="139"/>
+      <c r="AG4" s="139"/>
+      <c r="AH4" s="139"/>
+      <c r="AJ4" s="135"/>
+      <c r="AK4" s="135"/>
+      <c r="AL4" s="135"/>
+      <c r="AM4" s="135"/>
+      <c r="AN4" s="135"/>
+      <c r="AO4" s="135"/>
+      <c r="AP4" s="135"/>
     </row>
-    <row r="5" spans="1:68" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:68" ht="30" customHeight="1">
       <c r="A5" s="10" t="s">
         <v>34</v>
       </c>
@@ -2846,7 +2846,7 @@
       <c r="G5" s="72"/>
       <c r="H5" s="72"/>
     </row>
-    <row r="6" spans="1:68" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:68" ht="30" customHeight="1">
       <c r="A6" s="10"/>
       <c r="B6" s="76" t="s">
         <v>6</v>
@@ -2940,7 +2940,7 @@
       <c r="BK6" s="87"/>
       <c r="BL6" s="87"/>
     </row>
-    <row r="7" spans="1:68" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:68" ht="30" customHeight="1">
       <c r="A7" s="10"/>
       <c r="B7" s="76" t="s">
         <v>7</v>
@@ -3178,7 +3178,7 @@
         <v>46021</v>
       </c>
     </row>
-    <row r="8" spans="1:68" ht="19.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:68" ht="19.899999999999999" customHeight="1">
       <c r="A8" s="10"/>
       <c r="B8" s="71"/>
       <c r="C8" s="71"/>
@@ -3244,7 +3244,7 @@
       <c r="BK8" s="99"/>
       <c r="BL8" s="102"/>
     </row>
-    <row r="9" spans="1:68" ht="40.15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:68" ht="40.15" customHeight="1">
       <c r="A9" s="10" t="s">
         <v>35</v>
       </c>
@@ -3492,7 +3492,7 @@
         <v>D</v>
       </c>
     </row>
-    <row r="10" spans="1:68" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:68" ht="30" hidden="1" customHeight="1">
       <c r="B10" s="16"/>
       <c r="C10" s="13"/>
       <c r="D10" s="12"/>
@@ -3556,7 +3556,7 @@
       <c r="BK10" s="34"/>
       <c r="BL10" s="34"/>
     </row>
-    <row r="11" spans="1:68" s="1" customFormat="1" ht="40.15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:68" s="1" customFormat="1" ht="40.15" customHeight="1">
       <c r="A11" s="10"/>
       <c r="B11" s="123" t="s">
         <v>43</v>
@@ -3801,7 +3801,7 @@
       </c>
       <c r="BP11" s="39"/>
     </row>
-    <row r="12" spans="1:68" s="1" customFormat="1" ht="40.15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:68" s="1" customFormat="1" ht="40.15" customHeight="1">
       <c r="A12" s="10"/>
       <c r="B12" s="123"/>
       <c r="C12" s="57" t="s">
@@ -4043,7 +4043,7 @@
         <v/>
       </c>
     </row>
-    <row r="13" spans="1:68" s="1" customFormat="1" ht="40.15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:68" s="1" customFormat="1" ht="40.15" customHeight="1">
       <c r="A13" s="10"/>
       <c r="B13" s="123" t="s">
         <v>44</v>
@@ -4287,7 +4287,7 @@
         <v/>
       </c>
     </row>
-    <row r="14" spans="1:68" s="1" customFormat="1" ht="40.15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:68" s="1" customFormat="1" ht="40.15" customHeight="1">
       <c r="A14" s="9"/>
       <c r="B14" s="123"/>
       <c r="C14" s="57" t="s">
@@ -4529,7 +4529,7 @@
         <v/>
       </c>
     </row>
-    <row r="15" spans="1:68" s="1" customFormat="1" ht="40.15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:68" s="1" customFormat="1" ht="40.15" customHeight="1">
       <c r="A15" s="9"/>
       <c r="B15" s="123" t="s">
         <v>45</v>
@@ -4773,7 +4773,7 @@
         <v/>
       </c>
     </row>
-    <row r="16" spans="1:68" s="1" customFormat="1" ht="40.15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:68" s="1" customFormat="1" ht="40.15" customHeight="1">
       <c r="A16" s="9"/>
       <c r="B16" s="123"/>
       <c r="C16" s="57" t="s">
@@ -5015,7 +5015,7 @@
         <v/>
       </c>
     </row>
-    <row r="17" spans="1:64" s="1" customFormat="1" ht="40.15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:64" s="1" customFormat="1" ht="40.15" customHeight="1">
       <c r="A17" s="10"/>
       <c r="B17" s="123" t="s">
         <v>46</v>
@@ -5259,7 +5259,7 @@
         <v/>
       </c>
     </row>
-    <row r="18" spans="1:64" s="1" customFormat="1" ht="40.15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:64" s="1" customFormat="1" ht="40.15" customHeight="1">
       <c r="A18" s="10"/>
       <c r="B18" s="123"/>
       <c r="C18" s="57" t="s">
@@ -5501,7 +5501,7 @@
         <v/>
       </c>
     </row>
-    <row r="19" spans="1:64" s="1" customFormat="1" ht="40.15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:64" s="1" customFormat="1" ht="40.15" customHeight="1">
       <c r="A19" s="9"/>
       <c r="B19" s="123" t="s">
         <v>47</v>
@@ -5745,7 +5745,7 @@
         <v/>
       </c>
     </row>
-    <row r="20" spans="1:64" s="1" customFormat="1" ht="40.15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:64" s="1" customFormat="1" ht="40.15" customHeight="1">
       <c r="A20" s="9"/>
       <c r="B20" s="123"/>
       <c r="C20" s="57" t="s">
@@ -5987,7 +5987,7 @@
         <v/>
       </c>
     </row>
-    <row r="21" spans="1:64" s="1" customFormat="1" ht="40.15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:64" s="1" customFormat="1" ht="40.15" customHeight="1">
       <c r="A21" s="9"/>
       <c r="B21" s="123" t="s">
         <v>48</v>
@@ -6231,7 +6231,7 @@
         <v/>
       </c>
     </row>
-    <row r="22" spans="1:64" s="1" customFormat="1" ht="40.15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:64" s="1" customFormat="1" ht="40.15" customHeight="1">
       <c r="A22" s="9"/>
       <c r="B22" s="123"/>
       <c r="C22" s="57" t="s">
@@ -6473,7 +6473,7 @@
         <v/>
       </c>
     </row>
-    <row r="23" spans="1:64" s="1" customFormat="1" ht="40.15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:64" s="1" customFormat="1" ht="40.15" customHeight="1">
       <c r="A23" s="9"/>
       <c r="B23" s="123" t="s">
         <v>49</v>
@@ -6709,7 +6709,7 @@
         <v/>
       </c>
     </row>
-    <row r="24" spans="1:64" s="1" customFormat="1" ht="40.15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:64" s="1" customFormat="1" ht="40.15" customHeight="1">
       <c r="A24" s="9"/>
       <c r="B24" s="123"/>
       <c r="C24" s="57"/>
@@ -6943,7 +6943,7 @@
         <v/>
       </c>
     </row>
-    <row r="25" spans="1:64" s="1" customFormat="1" ht="40.15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:64" s="1" customFormat="1" ht="40.15" customHeight="1">
       <c r="A25" s="9"/>
       <c r="B25" s="123" t="s">
         <v>50</v>
@@ -7179,7 +7179,7 @@
         <v/>
       </c>
     </row>
-    <row r="26" spans="1:64" s="1" customFormat="1" ht="40.15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:64" s="1" customFormat="1" ht="40.15" customHeight="1">
       <c r="A26" s="9"/>
       <c r="B26" s="123"/>
       <c r="C26" s="57"/>
@@ -7413,7 +7413,7 @@
         <v/>
       </c>
     </row>
-    <row r="27" spans="1:64" s="1" customFormat="1" ht="40.15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:64" s="1" customFormat="1" ht="40.15" customHeight="1">
       <c r="A27" s="9"/>
       <c r="B27" s="123" t="s">
         <v>51</v>
@@ -7649,7 +7649,7 @@
         <v/>
       </c>
     </row>
-    <row r="28" spans="1:64" s="1" customFormat="1" ht="40.15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:64" s="1" customFormat="1" ht="40.15" customHeight="1">
       <c r="A28" s="9"/>
       <c r="B28" s="61"/>
       <c r="C28" s="57"/>
@@ -7883,7 +7883,7 @@
         <v/>
       </c>
     </row>
-    <row r="29" spans="1:64" s="1" customFormat="1" ht="40.15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:64" s="1" customFormat="1" ht="40.15" customHeight="1">
       <c r="A29" s="9"/>
       <c r="B29" s="113"/>
       <c r="C29" s="57"/>
@@ -8117,7 +8117,7 @@
         <v/>
       </c>
     </row>
-    <row r="30" spans="1:64" s="1" customFormat="1" ht="40.15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:64" s="1" customFormat="1" ht="40.15" customHeight="1">
       <c r="A30" s="9"/>
       <c r="B30" s="61"/>
       <c r="C30" s="57"/>
@@ -8351,7 +8351,7 @@
         <v/>
       </c>
     </row>
-    <row r="31" spans="1:64" s="1" customFormat="1" ht="40.15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:64" s="1" customFormat="1" ht="40.15" customHeight="1">
       <c r="A31" s="9"/>
       <c r="B31" s="61"/>
       <c r="C31" s="57"/>
@@ -8585,7 +8585,7 @@
         <v/>
       </c>
     </row>
-    <row r="32" spans="1:64" s="1" customFormat="1" ht="40.15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:64" s="1" customFormat="1" ht="40.15" customHeight="1">
       <c r="A32" s="9"/>
       <c r="B32" s="61"/>
       <c r="C32" s="57"/>
@@ -8819,7 +8819,7 @@
         <v/>
       </c>
     </row>
-    <row r="33" spans="1:65" s="1" customFormat="1" ht="40.15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:65" s="1" customFormat="1" ht="40.15" customHeight="1">
       <c r="A33" s="9"/>
       <c r="B33" s="61"/>
       <c r="C33" s="57"/>
@@ -9053,7 +9053,7 @@
         <v/>
       </c>
     </row>
-    <row r="34" spans="1:65" s="1" customFormat="1" ht="40.15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:65" s="1" customFormat="1" ht="40.15" customHeight="1">
       <c r="A34" s="9"/>
       <c r="B34" s="61"/>
       <c r="C34" s="57"/>
@@ -9287,7 +9287,7 @@
         <v/>
       </c>
     </row>
-    <row r="35" spans="1:65" s="1" customFormat="1" ht="40.15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:65" s="1" customFormat="1" ht="40.15" customHeight="1">
       <c r="A35" s="9"/>
       <c r="B35" s="61"/>
       <c r="C35" s="57"/>
@@ -9522,7 +9522,7 @@
       </c>
       <c r="BM35" s="86"/>
     </row>
-    <row r="36" spans="1:65" s="1" customFormat="1" ht="40.15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:65" s="1" customFormat="1" ht="40.15" customHeight="1">
       <c r="A36" s="10"/>
       <c r="B36" s="115" t="s">
         <v>18</v>
@@ -9590,12 +9590,12 @@
       <c r="BK36" s="84"/>
       <c r="BL36" s="84"/>
     </row>
-    <row r="37" spans="1:65" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:65" ht="30" customHeight="1">
       <c r="D37" s="4"/>
       <c r="G37" s="11"/>
       <c r="H37" s="3"/>
     </row>
-    <row r="38" spans="1:65" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:65" ht="30" customHeight="1">
       <c r="D38" s="5"/>
     </row>
   </sheetData>
@@ -9755,7 +9755,7 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:BP38"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="30" customHeight="1" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="30" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="4.7109375" style="9" customWidth="1"/>
     <col min="2" max="2" width="37.85546875" customWidth="1"/>
@@ -9769,30 +9769,30 @@
     <col min="65" max="65" width="2.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:68" ht="25.15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="2" spans="1:68" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:68" ht="25.15" customHeight="1"/>
+    <row r="2" spans="1:68" ht="49.9" customHeight="1">
       <c r="A2" s="10"/>
-      <c r="B2" s="133" t="s">
+      <c r="B2" s="125" t="s">
         <v>3</v>
       </c>
-      <c r="C2" s="133"/>
-      <c r="D2" s="133"/>
-      <c r="E2" s="133"/>
-      <c r="F2" s="133"/>
-      <c r="G2" s="133"/>
-      <c r="H2" s="133"/>
-      <c r="I2" s="134"/>
-      <c r="J2" s="134"/>
-      <c r="K2" s="134"/>
-      <c r="L2" s="134"/>
-      <c r="M2" s="134"/>
-      <c r="N2" s="134"/>
-      <c r="O2" s="135"/>
-      <c r="P2" s="136"/>
-      <c r="Q2" s="136"/>
-      <c r="R2" s="136"/>
-      <c r="S2" s="136"/>
-      <c r="T2" s="136"/>
+      <c r="C2" s="125"/>
+      <c r="D2" s="125"/>
+      <c r="E2" s="125"/>
+      <c r="F2" s="125"/>
+      <c r="G2" s="125"/>
+      <c r="H2" s="125"/>
+      <c r="I2" s="126"/>
+      <c r="J2" s="126"/>
+      <c r="K2" s="126"/>
+      <c r="L2" s="126"/>
+      <c r="M2" s="126"/>
+      <c r="N2" s="126"/>
+      <c r="O2" s="127"/>
+      <c r="P2" s="128"/>
+      <c r="Q2" s="128"/>
+      <c r="R2" s="128"/>
+      <c r="S2" s="128"/>
+      <c r="T2" s="128"/>
       <c r="U2" s="20"/>
       <c r="V2" s="20"/>
       <c r="W2" s="20"/>
@@ -9839,7 +9839,7 @@
       <c r="BL2" s="20"/>
       <c r="BM2" s="20"/>
     </row>
-    <row r="3" spans="1:68" ht="19.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:68" ht="19.899999999999999" customHeight="1">
       <c r="A3" s="10"/>
       <c r="B3" s="40"/>
       <c r="C3" s="41"/>
@@ -9906,7 +9906,7 @@
       <c r="BL3" s="30"/>
       <c r="BM3" s="30"/>
     </row>
-    <row r="4" spans="1:68" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:68" ht="30" customHeight="1">
       <c r="A4" s="10"/>
       <c r="B4" s="52" t="s">
         <v>36</v>
@@ -9919,50 +9919,50 @@
         <v>30</v>
       </c>
       <c r="H4" s="27"/>
-      <c r="I4" s="130" t="s">
+      <c r="I4" s="129" t="s">
         <v>41</v>
       </c>
-      <c r="J4" s="130"/>
-      <c r="K4" s="130"/>
-      <c r="L4" s="130"/>
-      <c r="M4" s="130"/>
-      <c r="N4" s="130"/>
+      <c r="J4" s="129"/>
+      <c r="K4" s="129"/>
+      <c r="L4" s="129"/>
+      <c r="M4" s="129"/>
+      <c r="N4" s="129"/>
       <c r="O4" s="30"/>
-      <c r="P4" s="137" t="s">
+      <c r="P4" s="130" t="s">
         <v>42</v>
       </c>
-      <c r="Q4" s="137"/>
-      <c r="R4" s="137"/>
-      <c r="S4" s="137"/>
-      <c r="T4" s="137"/>
-      <c r="U4" s="137"/>
+      <c r="Q4" s="130"/>
+      <c r="R4" s="130"/>
+      <c r="S4" s="130"/>
+      <c r="T4" s="130"/>
+      <c r="U4" s="130"/>
       <c r="V4" s="30"/>
-      <c r="W4" s="138" t="s">
+      <c r="W4" s="131" t="s">
         <v>33</v>
       </c>
-      <c r="X4" s="138"/>
-      <c r="Y4" s="138"/>
-      <c r="Z4" s="138"/>
-      <c r="AA4" s="138"/>
-      <c r="AB4" s="138"/>
+      <c r="X4" s="131"/>
+      <c r="Y4" s="131"/>
+      <c r="Z4" s="131"/>
+      <c r="AA4" s="131"/>
+      <c r="AB4" s="131"/>
       <c r="AC4" s="30"/>
-      <c r="AD4" s="139" t="s">
+      <c r="AD4" s="132" t="s">
         <v>33</v>
       </c>
-      <c r="AE4" s="139"/>
-      <c r="AF4" s="139"/>
-      <c r="AG4" s="139"/>
-      <c r="AH4" s="139"/>
+      <c r="AE4" s="132"/>
+      <c r="AF4" s="132"/>
+      <c r="AG4" s="132"/>
+      <c r="AH4" s="132"/>
       <c r="AI4" s="30"/>
-      <c r="AJ4" s="132" t="s">
+      <c r="AJ4" s="124" t="s">
         <v>33</v>
       </c>
-      <c r="AK4" s="132"/>
-      <c r="AL4" s="132"/>
-      <c r="AM4" s="132"/>
-      <c r="AN4" s="132"/>
-      <c r="AO4" s="132"/>
-      <c r="AP4" s="132"/>
+      <c r="AK4" s="124"/>
+      <c r="AL4" s="124"/>
+      <c r="AM4" s="124"/>
+      <c r="AN4" s="124"/>
+      <c r="AO4" s="124"/>
+      <c r="AP4" s="124"/>
       <c r="AQ4" s="30"/>
       <c r="AR4" s="30"/>
       <c r="AS4" s="30"/>
@@ -9987,7 +9987,7 @@
       <c r="BL4" s="30"/>
       <c r="BM4" s="30"/>
     </row>
-    <row r="5" spans="1:68" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:68" ht="30" customHeight="1">
       <c r="A5" s="10" t="s">
         <v>34</v>
       </c>
@@ -10058,7 +10058,7 @@
       <c r="BL5" s="30"/>
       <c r="BM5" s="30"/>
     </row>
-    <row r="6" spans="1:68" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:68" ht="30" customHeight="1">
       <c r="A6" s="10"/>
       <c r="B6" s="47" t="s">
         <v>6</v>
@@ -10153,7 +10153,7 @@
       <c r="BL6" s="63"/>
       <c r="BM6" s="30"/>
     </row>
-    <row r="7" spans="1:68" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:68" ht="30" customHeight="1">
       <c r="A7" s="10"/>
       <c r="B7" s="47" t="s">
         <v>7</v>
@@ -10392,7 +10392,7 @@
       </c>
       <c r="BM7" s="30"/>
     </row>
-    <row r="8" spans="1:68" ht="19.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:68" ht="19.899999999999999" customHeight="1">
       <c r="A8" s="10"/>
       <c r="B8" s="49"/>
       <c r="C8" s="49"/>
@@ -10459,7 +10459,7 @@
       <c r="BL8" s="37"/>
       <c r="BM8" s="30"/>
     </row>
-    <row r="9" spans="1:68" ht="40.15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:68" ht="40.15" customHeight="1">
       <c r="A9" s="10" t="s">
         <v>35</v>
       </c>
@@ -10708,7 +10708,7 @@
       </c>
       <c r="BM9" s="30"/>
     </row>
-    <row r="10" spans="1:68" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:68" ht="30" hidden="1" customHeight="1">
       <c r="B10" s="16"/>
       <c r="C10" s="13"/>
       <c r="D10" s="12"/>
@@ -10774,7 +10774,7 @@
       <c r="BL10" s="34"/>
       <c r="BM10" s="30"/>
     </row>
-    <row r="11" spans="1:68" s="1" customFormat="1" ht="40.15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:68" s="1" customFormat="1" ht="40.15" customHeight="1">
       <c r="A11" s="10"/>
       <c r="B11" s="120" t="s">
         <v>38</v>
@@ -11015,7 +11015,7 @@
       </c>
       <c r="BP11" s="39"/>
     </row>
-    <row r="12" spans="1:68" s="1" customFormat="1" ht="40.15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:68" s="1" customFormat="1" ht="40.15" customHeight="1">
       <c r="A12" s="10"/>
       <c r="B12" s="121" t="s">
         <v>53</v>
@@ -11261,7 +11261,7 @@
         <v/>
       </c>
     </row>
-    <row r="13" spans="1:68" s="1" customFormat="1" ht="40.15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:68" s="1" customFormat="1" ht="40.15" customHeight="1">
       <c r="A13" s="10"/>
       <c r="B13" s="121"/>
       <c r="C13" s="21" t="s">
@@ -11505,7 +11505,7 @@
         <v/>
       </c>
     </row>
-    <row r="14" spans="1:68" s="1" customFormat="1" ht="40.15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:68" s="1" customFormat="1" ht="40.15" customHeight="1">
       <c r="A14" s="9"/>
       <c r="B14" s="121" t="s">
         <v>54</v>
@@ -11751,7 +11751,7 @@
         <v/>
       </c>
     </row>
-    <row r="15" spans="1:68" s="1" customFormat="1" ht="40.15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:68" s="1" customFormat="1" ht="40.15" customHeight="1">
       <c r="A15" s="9"/>
       <c r="B15" s="121"/>
       <c r="C15" s="21" t="s">
@@ -11995,7 +11995,7 @@
         <v/>
       </c>
     </row>
-    <row r="16" spans="1:68" s="1" customFormat="1" ht="40.15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:68" s="1" customFormat="1" ht="40.15" customHeight="1">
       <c r="A16" s="9"/>
       <c r="B16" s="121" t="s">
         <v>55</v>
@@ -12241,7 +12241,7 @@
         <v/>
       </c>
     </row>
-    <row r="17" spans="1:65" s="1" customFormat="1" ht="40.15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:65" s="1" customFormat="1" ht="40.15" customHeight="1">
       <c r="A17" s="10"/>
       <c r="B17" s="121"/>
       <c r="C17" s="21" t="s">
@@ -12485,7 +12485,7 @@
         <v/>
       </c>
     </row>
-    <row r="18" spans="1:65" s="1" customFormat="1" ht="40.15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:65" s="1" customFormat="1" ht="40.15" customHeight="1">
       <c r="A18" s="10"/>
       <c r="B18" s="121" t="s">
         <v>56</v>
@@ -12731,7 +12731,7 @@
         <v/>
       </c>
     </row>
-    <row r="19" spans="1:65" s="1" customFormat="1" ht="40.15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:65" s="1" customFormat="1" ht="40.15" customHeight="1">
       <c r="A19" s="9"/>
       <c r="B19" s="12"/>
       <c r="C19" s="21" t="s">
@@ -12975,7 +12975,7 @@
         <v/>
       </c>
     </row>
-    <row r="20" spans="1:65" s="1" customFormat="1" ht="40.15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:65" s="1" customFormat="1" ht="40.15" customHeight="1">
       <c r="A20" s="9"/>
       <c r="B20" s="121" t="s">
         <v>57</v>
@@ -13221,7 +13221,7 @@
         <v/>
       </c>
     </row>
-    <row r="21" spans="1:65" s="1" customFormat="1" ht="40.15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:65" s="1" customFormat="1" ht="40.15" customHeight="1">
       <c r="A21" s="9"/>
       <c r="B21" s="121"/>
       <c r="C21" s="21" t="s">
@@ -13461,7 +13461,7 @@
         <v/>
       </c>
     </row>
-    <row r="22" spans="1:65" s="1" customFormat="1" ht="40.15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:65" s="1" customFormat="1" ht="40.15" customHeight="1">
       <c r="A22" s="9"/>
       <c r="B22" s="121"/>
       <c r="C22" s="21" t="s">
@@ -13701,7 +13701,7 @@
         <v/>
       </c>
     </row>
-    <row r="23" spans="1:65" s="1" customFormat="1" ht="40.15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:65" s="1" customFormat="1" ht="40.15" customHeight="1">
       <c r="A23" s="9"/>
       <c r="B23" s="121"/>
       <c r="C23" s="21" t="s">
@@ -13941,7 +13941,7 @@
         <v/>
       </c>
     </row>
-    <row r="24" spans="1:65" s="1" customFormat="1" ht="40.15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:65" s="1" customFormat="1" ht="40.15" customHeight="1">
       <c r="A24" s="9"/>
       <c r="B24" s="121"/>
       <c r="C24" s="21" t="s">
@@ -14181,7 +14181,7 @@
         <v/>
       </c>
     </row>
-    <row r="25" spans="1:65" s="1" customFormat="1" ht="40.15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:65" s="1" customFormat="1" ht="40.15" customHeight="1">
       <c r="A25" s="9"/>
       <c r="B25" s="121"/>
       <c r="C25" s="21" t="s">
@@ -14421,7 +14421,7 @@
         <v/>
       </c>
     </row>
-    <row r="26" spans="1:65" s="1" customFormat="1" ht="40.15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:65" s="1" customFormat="1" ht="40.15" customHeight="1">
       <c r="A26" s="9"/>
       <c r="B26" s="121"/>
       <c r="C26" s="21" t="s">
@@ -14661,7 +14661,7 @@
         <v/>
       </c>
     </row>
-    <row r="27" spans="1:65" s="1" customFormat="1" ht="40.15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:65" s="1" customFormat="1" ht="40.15" customHeight="1">
       <c r="A27" s="9"/>
       <c r="B27" s="121"/>
       <c r="C27" s="21" t="s">
@@ -14901,7 +14901,7 @@
         <v/>
       </c>
     </row>
-    <row r="28" spans="1:65" s="1" customFormat="1" ht="40.15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:65" s="1" customFormat="1" ht="40.15" customHeight="1">
       <c r="A28" s="9"/>
       <c r="B28" s="12"/>
       <c r="C28" s="21" t="s">
@@ -15141,7 +15141,7 @@
         <v/>
       </c>
     </row>
-    <row r="29" spans="1:65" s="1" customFormat="1" ht="40.15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:65" s="1" customFormat="1" ht="40.15" customHeight="1">
       <c r="A29" s="9"/>
       <c r="B29" s="121"/>
       <c r="C29" s="21" t="s">
@@ -15381,7 +15381,7 @@
         <v/>
       </c>
     </row>
-    <row r="30" spans="1:65" s="1" customFormat="1" ht="40.15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:65" s="1" customFormat="1" ht="40.15" customHeight="1">
       <c r="A30" s="9"/>
       <c r="B30" s="121"/>
       <c r="C30" s="21" t="s">
@@ -15621,7 +15621,7 @@
         <v/>
       </c>
     </row>
-    <row r="31" spans="1:65" s="1" customFormat="1" ht="40.15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:65" s="1" customFormat="1" ht="40.15" customHeight="1">
       <c r="A31" s="9"/>
       <c r="B31" s="121"/>
       <c r="C31" s="21" t="s">
@@ -15861,7 +15861,7 @@
         <v/>
       </c>
     </row>
-    <row r="32" spans="1:65" s="1" customFormat="1" ht="40.15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:65" s="1" customFormat="1" ht="40.15" customHeight="1">
       <c r="A32" s="9"/>
       <c r="B32" s="121"/>
       <c r="C32" s="21" t="s">
@@ -16101,7 +16101,7 @@
         <v/>
       </c>
     </row>
-    <row r="33" spans="1:65" s="1" customFormat="1" ht="40.15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:65" s="1" customFormat="1" ht="40.15" customHeight="1">
       <c r="A33" s="9"/>
       <c r="B33" s="121"/>
       <c r="C33" s="21" t="s">
@@ -16341,7 +16341,7 @@
         <v/>
       </c>
     </row>
-    <row r="34" spans="1:65" s="1" customFormat="1" ht="40.15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:65" s="1" customFormat="1" ht="40.15" customHeight="1">
       <c r="A34" s="9"/>
       <c r="B34" s="121"/>
       <c r="C34" s="21" t="s">
@@ -16581,7 +16581,7 @@
         <v/>
       </c>
     </row>
-    <row r="35" spans="1:65" s="1" customFormat="1" ht="40.15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:65" s="1" customFormat="1" ht="40.15" customHeight="1">
       <c r="A35" s="9"/>
       <c r="B35" s="121"/>
       <c r="C35" s="21" t="s">
@@ -16821,7 +16821,7 @@
         <v/>
       </c>
     </row>
-    <row r="36" spans="1:65" s="1" customFormat="1" ht="40.15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:65" s="1" customFormat="1" ht="40.15" customHeight="1">
       <c r="A36" s="10"/>
       <c r="B36" s="114" t="s">
         <v>18</v>
@@ -16890,12 +16890,12 @@
       <c r="BL36" s="54"/>
       <c r="BM36" s="26"/>
     </row>
-    <row r="37" spans="1:65" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:65" ht="30" customHeight="1">
       <c r="D37" s="4"/>
       <c r="G37" s="11"/>
       <c r="H37" s="3"/>
     </row>
-    <row r="38" spans="1:65" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:65" ht="30" customHeight="1">
       <c r="D38" s="5"/>
     </row>
   </sheetData>
@@ -17059,7 +17059,7 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:BP38"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="30" customHeight="1" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="30" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="4.7109375" style="9" customWidth="1"/>
     <col min="2" max="2" width="37.85546875" customWidth="1"/>
@@ -17073,8 +17073,8 @@
     <col min="65" max="65" width="2.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:68" ht="25.15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="2" spans="1:68" ht="49.9" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:68" ht="25.15" customHeight="1"/>
+    <row r="2" spans="1:68" ht="49.9" customHeight="1">
       <c r="A2" s="10"/>
       <c r="B2" s="140" t="s">
         <v>3</v>
@@ -17143,7 +17143,7 @@
       <c r="BL2" s="94"/>
       <c r="BM2" s="94"/>
     </row>
-    <row r="3" spans="1:68" ht="19.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:68" ht="19.899999999999999" customHeight="1">
       <c r="A3" s="10"/>
       <c r="B3" s="65"/>
       <c r="C3" s="66"/>
@@ -17157,7 +17157,7 @@
       <c r="K3" s="1"/>
       <c r="L3" s="1"/>
     </row>
-    <row r="4" spans="1:68" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:68" ht="30" customHeight="1">
       <c r="A4" s="10"/>
       <c r="B4" s="69" t="s">
         <v>4</v>
@@ -17170,48 +17170,48 @@
         <v>30</v>
       </c>
       <c r="H4" s="72"/>
-      <c r="I4" s="130" t="s">
+      <c r="I4" s="129" t="s">
         <v>25</v>
       </c>
-      <c r="J4" s="130"/>
-      <c r="K4" s="130"/>
-      <c r="L4" s="130"/>
-      <c r="M4" s="130"/>
-      <c r="N4" s="130"/>
-      <c r="P4" s="137" t="s">
+      <c r="J4" s="129"/>
+      <c r="K4" s="129"/>
+      <c r="L4" s="129"/>
+      <c r="M4" s="129"/>
+      <c r="N4" s="129"/>
+      <c r="P4" s="130" t="s">
         <v>22</v>
       </c>
-      <c r="Q4" s="137"/>
-      <c r="R4" s="137"/>
-      <c r="S4" s="137"/>
-      <c r="T4" s="137"/>
-      <c r="U4" s="137"/>
-      <c r="W4" s="138" t="s">
+      <c r="Q4" s="130"/>
+      <c r="R4" s="130"/>
+      <c r="S4" s="130"/>
+      <c r="T4" s="130"/>
+      <c r="U4" s="130"/>
+      <c r="W4" s="131" t="s">
         <v>23</v>
       </c>
-      <c r="X4" s="138"/>
-      <c r="Y4" s="138"/>
-      <c r="Z4" s="138"/>
-      <c r="AA4" s="138"/>
-      <c r="AB4" s="138"/>
-      <c r="AD4" s="139" t="s">
+      <c r="X4" s="131"/>
+      <c r="Y4" s="131"/>
+      <c r="Z4" s="131"/>
+      <c r="AA4" s="131"/>
+      <c r="AB4" s="131"/>
+      <c r="AD4" s="132" t="s">
         <v>32</v>
       </c>
-      <c r="AE4" s="139"/>
-      <c r="AF4" s="139"/>
-      <c r="AG4" s="139"/>
-      <c r="AH4" s="139"/>
-      <c r="AJ4" s="132" t="s">
+      <c r="AE4" s="132"/>
+      <c r="AF4" s="132"/>
+      <c r="AG4" s="132"/>
+      <c r="AH4" s="132"/>
+      <c r="AJ4" s="124" t="s">
         <v>33</v>
       </c>
-      <c r="AK4" s="132"/>
-      <c r="AL4" s="132"/>
-      <c r="AM4" s="132"/>
-      <c r="AN4" s="132"/>
-      <c r="AO4" s="132"/>
-      <c r="AP4" s="132"/>
+      <c r="AK4" s="124"/>
+      <c r="AL4" s="124"/>
+      <c r="AM4" s="124"/>
+      <c r="AN4" s="124"/>
+      <c r="AO4" s="124"/>
+      <c r="AP4" s="124"/>
     </row>
-    <row r="5" spans="1:68" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:68" ht="30" customHeight="1">
       <c r="A5" s="10" t="s">
         <v>34</v>
       </c>
@@ -17225,14 +17225,14 @@
       <c r="G5" s="72"/>
       <c r="H5" s="72"/>
     </row>
-    <row r="6" spans="1:68" ht="30" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:68" ht="30" customHeight="1">
       <c r="A6" s="10"/>
       <c r="B6" s="76" t="s">
         <v>6</v>
       </c>
       <c r="C6" s="77" cm="1">
         <f t="array" aca="1" ref="C6" ca="1">IFERROR(IF(MIN(Meilensteine43524[Start])=0,TODAY(),B11(Meilensteine43524[Start])),TODAY())</f>
-        <v>46035</v>
+        <v>46070</v>
       </c>
       <c r="D6" s="78"/>
       <c r="E6" s="72"/>
@@ -17241,7 +17241,7 @@
       <c r="H6" s="72"/>
       <c r="I6" s="88" t="str">
         <f ca="1">TEXT(I7,"MMMM")</f>
-        <v>Januar</v>
+        <v>Februar</v>
       </c>
       <c r="J6" s="88"/>
       <c r="K6" s="88"/>
@@ -17261,7 +17261,7 @@
       <c r="V6" s="88"/>
       <c r="W6" s="88" t="str">
         <f ca="1">IF(OR(TEXT(W7,"MMMM")=P6,TEXT(W7,"MMMM")=I6),"",TEXT(W7,"MMMM"))</f>
-        <v/>
+        <v>März</v>
       </c>
       <c r="X6" s="88"/>
       <c r="Y6" s="88"/>
@@ -17271,7 +17271,7 @@
       <c r="AC6" s="88"/>
       <c r="AD6" s="88" t="str">
         <f ca="1">IF(OR(TEXT(AD7,"MMMM")=W6,TEXT(AD7,"MMMM")=P6,TEXT(AD7,"MMMM")=I6),"",TEXT(AD7,"MMMM"))</f>
-        <v>Februar</v>
+        <v/>
       </c>
       <c r="AE6" s="88"/>
       <c r="AF6" s="88"/>
@@ -17301,7 +17301,7 @@
       <c r="AX6" s="89"/>
       <c r="AY6" s="89" t="str">
         <f ca="1">IF(OR(TEXT(AY7,"MMMM")=AR6,TEXT(AY7,"MMMM")=AK6,TEXT(AY7,"MMMM")=AD6,TEXT(AY7,"MMMM")=W6),"",TEXT(AY7,"MMMM"))</f>
-        <v/>
+        <v>April</v>
       </c>
       <c r="AZ6" s="89"/>
       <c r="BA6" s="89"/>
@@ -17311,7 +17311,7 @@
       <c r="BE6" s="87"/>
       <c r="BF6" s="87" t="str">
         <f ca="1">IF(OR(TEXT(BF7,"MMMM")=AY6,TEXT(BF7,"MMMM")=AR6,TEXT(BF7,"MMMM")=AK6,TEXT(BF7,"MMMM")=AD6),"",TEXT(BF7,"MMMM"))</f>
-        <v>März</v>
+        <v/>
       </c>
       <c r="BG6" s="87"/>
       <c r="BH6" s="87"/>
@@ -17320,7 +17320,7 @@
       <c r="BK6" s="87"/>
       <c r="BL6" s="87"/>
     </row>
-    <row r="7" spans="1:68" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:68" ht="30" customHeight="1">
       <c r="A7" s="10"/>
       <c r="B7" s="76" t="s">
         <v>7</v>
@@ -17335,230 +17335,230 @@
       <c r="H7" s="80"/>
       <c r="I7" s="95">
         <f ca="1">IFERROR(Projekt_Start+Scrollschrittweite,TODAY())</f>
-        <v>46036</v>
+        <v>46071</v>
       </c>
       <c r="J7" s="96">
         <f ca="1">I7+1</f>
-        <v>46037</v>
+        <v>46072</v>
       </c>
       <c r="K7" s="96">
         <f t="shared" ref="K7:AX7" ca="1" si="0">J7+1</f>
-        <v>46038</v>
+        <v>46073</v>
       </c>
       <c r="L7" s="96">
         <f t="shared" ca="1" si="0"/>
-        <v>46039</v>
+        <v>46074</v>
       </c>
       <c r="M7" s="96">
         <f t="shared" ca="1" si="0"/>
-        <v>46040</v>
+        <v>46075</v>
       </c>
       <c r="N7" s="96">
         <f t="shared" ca="1" si="0"/>
-        <v>46041</v>
+        <v>46076</v>
       </c>
       <c r="O7" s="97">
         <f t="shared" ca="1" si="0"/>
-        <v>46042</v>
+        <v>46077</v>
       </c>
       <c r="P7" s="96">
         <f ca="1">O7+1</f>
-        <v>46043</v>
+        <v>46078</v>
       </c>
       <c r="Q7" s="96">
         <f ca="1">P7+1</f>
-        <v>46044</v>
+        <v>46079</v>
       </c>
       <c r="R7" s="96">
         <f t="shared" ca="1" si="0"/>
-        <v>46045</v>
+        <v>46080</v>
       </c>
       <c r="S7" s="96">
         <f t="shared" ca="1" si="0"/>
-        <v>46046</v>
+        <v>46081</v>
       </c>
       <c r="T7" s="96">
         <f t="shared" ca="1" si="0"/>
-        <v>46047</v>
+        <v>46082</v>
       </c>
       <c r="U7" s="96">
         <f t="shared" ca="1" si="0"/>
-        <v>46048</v>
+        <v>46083</v>
       </c>
       <c r="V7" s="97">
         <f t="shared" ca="1" si="0"/>
-        <v>46049</v>
+        <v>46084</v>
       </c>
       <c r="W7" s="96">
         <f ca="1">V7+1</f>
-        <v>46050</v>
+        <v>46085</v>
       </c>
       <c r="X7" s="96">
         <f ca="1">W7+1</f>
-        <v>46051</v>
+        <v>46086</v>
       </c>
       <c r="Y7" s="96">
         <f t="shared" ca="1" si="0"/>
-        <v>46052</v>
+        <v>46087</v>
       </c>
       <c r="Z7" s="96">
         <f t="shared" ca="1" si="0"/>
-        <v>46053</v>
+        <v>46088</v>
       </c>
       <c r="AA7" s="96">
         <f t="shared" ca="1" si="0"/>
-        <v>46054</v>
+        <v>46089</v>
       </c>
       <c r="AB7" s="96">
         <f t="shared" ca="1" si="0"/>
-        <v>46055</v>
+        <v>46090</v>
       </c>
       <c r="AC7" s="97">
         <f t="shared" ca="1" si="0"/>
-        <v>46056</v>
+        <v>46091</v>
       </c>
       <c r="AD7" s="96">
         <f ca="1">AC7+1</f>
-        <v>46057</v>
+        <v>46092</v>
       </c>
       <c r="AE7" s="96">
         <f ca="1">AD7+1</f>
-        <v>46058</v>
+        <v>46093</v>
       </c>
       <c r="AF7" s="96">
         <f t="shared" ca="1" si="0"/>
-        <v>46059</v>
+        <v>46094</v>
       </c>
       <c r="AG7" s="96">
         <f t="shared" ca="1" si="0"/>
-        <v>46060</v>
+        <v>46095</v>
       </c>
       <c r="AH7" s="96">
         <f t="shared" ca="1" si="0"/>
-        <v>46061</v>
+        <v>46096</v>
       </c>
       <c r="AI7" s="96">
         <f t="shared" ca="1" si="0"/>
-        <v>46062</v>
+        <v>46097</v>
       </c>
       <c r="AJ7" s="97">
         <f t="shared" ca="1" si="0"/>
-        <v>46063</v>
+        <v>46098</v>
       </c>
       <c r="AK7" s="96">
         <f ca="1">AJ7+1</f>
-        <v>46064</v>
+        <v>46099</v>
       </c>
       <c r="AL7" s="96">
         <f ca="1">AK7+1</f>
-        <v>46065</v>
+        <v>46100</v>
       </c>
       <c r="AM7" s="96">
         <f t="shared" ca="1" si="0"/>
-        <v>46066</v>
+        <v>46101</v>
       </c>
       <c r="AN7" s="96">
         <f t="shared" ca="1" si="0"/>
-        <v>46067</v>
+        <v>46102</v>
       </c>
       <c r="AO7" s="96">
         <f t="shared" ca="1" si="0"/>
-        <v>46068</v>
+        <v>46103</v>
       </c>
       <c r="AP7" s="96">
         <f t="shared" ca="1" si="0"/>
-        <v>46069</v>
+        <v>46104</v>
       </c>
       <c r="AQ7" s="97">
         <f t="shared" ca="1" si="0"/>
-        <v>46070</v>
+        <v>46105</v>
       </c>
       <c r="AR7" s="96">
         <f ca="1">AQ7+1</f>
-        <v>46071</v>
+        <v>46106</v>
       </c>
       <c r="AS7" s="96">
         <f ca="1">AR7+1</f>
-        <v>46072</v>
+        <v>46107</v>
       </c>
       <c r="AT7" s="96">
         <f t="shared" ca="1" si="0"/>
-        <v>46073</v>
+        <v>46108</v>
       </c>
       <c r="AU7" s="96">
         <f t="shared" ca="1" si="0"/>
-        <v>46074</v>
+        <v>46109</v>
       </c>
       <c r="AV7" s="96">
         <f t="shared" ca="1" si="0"/>
-        <v>46075</v>
+        <v>46110</v>
       </c>
       <c r="AW7" s="96">
         <f t="shared" ca="1" si="0"/>
-        <v>46076</v>
+        <v>46111</v>
       </c>
       <c r="AX7" s="97">
         <f t="shared" ca="1" si="0"/>
-        <v>46077</v>
+        <v>46112</v>
       </c>
       <c r="AY7" s="96">
         <f ca="1">AX7+1</f>
-        <v>46078</v>
+        <v>46113</v>
       </c>
       <c r="AZ7" s="96">
         <f ca="1">AY7+1</f>
-        <v>46079</v>
+        <v>46114</v>
       </c>
       <c r="BA7" s="96">
         <f t="shared" ref="BA7:BE7" ca="1" si="1">AZ7+1</f>
-        <v>46080</v>
+        <v>46115</v>
       </c>
       <c r="BB7" s="96">
         <f t="shared" ca="1" si="1"/>
-        <v>46081</v>
+        <v>46116</v>
       </c>
       <c r="BC7" s="96">
         <f t="shared" ca="1" si="1"/>
-        <v>46082</v>
+        <v>46117</v>
       </c>
       <c r="BD7" s="96">
         <f t="shared" ca="1" si="1"/>
-        <v>46083</v>
+        <v>46118</v>
       </c>
       <c r="BE7" s="97">
         <f t="shared" ca="1" si="1"/>
-        <v>46084</v>
+        <v>46119</v>
       </c>
       <c r="BF7" s="96">
         <f ca="1">BE7+1</f>
-        <v>46085</v>
+        <v>46120</v>
       </c>
       <c r="BG7" s="96">
         <f ca="1">BF7+1</f>
-        <v>46086</v>
+        <v>46121</v>
       </c>
       <c r="BH7" s="96">
         <f t="shared" ref="BH7:BL7" ca="1" si="2">BG7+1</f>
-        <v>46087</v>
+        <v>46122</v>
       </c>
       <c r="BI7" s="96">
         <f t="shared" ca="1" si="2"/>
-        <v>46088</v>
+        <v>46123</v>
       </c>
       <c r="BJ7" s="96">
         <f t="shared" ca="1" si="2"/>
-        <v>46089</v>
+        <v>46124</v>
       </c>
       <c r="BK7" s="96">
         <f t="shared" ca="1" si="2"/>
-        <v>46090</v>
+        <v>46125</v>
       </c>
       <c r="BL7" s="97">
         <f t="shared" ca="1" si="2"/>
-        <v>46091</v>
+        <v>46126</v>
       </c>
     </row>
-    <row r="8" spans="1:68" ht="19.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:68" ht="19.899999999999999" customHeight="1">
       <c r="A8" s="10"/>
       <c r="B8" s="71"/>
       <c r="C8" s="71"/>
@@ -17624,7 +17624,7 @@
       <c r="BK8" s="99"/>
       <c r="BL8" s="102"/>
     </row>
-    <row r="9" spans="1:68" ht="40.15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:68" ht="40.15" customHeight="1">
       <c r="A9" s="10" t="s">
         <v>35</v>
       </c>
@@ -17872,7 +17872,7 @@
         <v>D</v>
       </c>
     </row>
-    <row r="10" spans="1:68" ht="30" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:68" ht="30" hidden="1" customHeight="1">
       <c r="B10" s="16"/>
       <c r="C10" s="13"/>
       <c r="D10" s="12"/>
@@ -17936,7 +17936,7 @@
       <c r="BK10" s="34"/>
       <c r="BL10" s="34"/>
     </row>
-    <row r="11" spans="1:68" s="1" customFormat="1" ht="40.15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:68" s="1" customFormat="1" ht="40.15" customHeight="1">
       <c r="A11" s="10"/>
       <c r="B11" s="113" t="s">
         <v>9</v>
@@ -18173,7 +18173,7 @@
       </c>
       <c r="BP11" s="39"/>
     </row>
-    <row r="12" spans="1:68" s="1" customFormat="1" ht="40.15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:68" s="1" customFormat="1" ht="40.15" customHeight="1">
       <c r="A12" s="10"/>
       <c r="B12" s="61" t="s">
         <v>10</v>
@@ -18189,7 +18189,7 @@
       </c>
       <c r="F12" s="59">
         <f ca="1">TODAY()</f>
-        <v>46035</v>
+        <v>46070</v>
       </c>
       <c r="G12" s="60">
         <v>3</v>
@@ -18420,7 +18420,7 @@
         <v/>
       </c>
     </row>
-    <row r="13" spans="1:68" s="1" customFormat="1" ht="40.15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:68" s="1" customFormat="1" ht="40.15" customHeight="1">
       <c r="A13" s="10"/>
       <c r="B13" s="61" t="s">
         <v>11</v>
@@ -18432,7 +18432,7 @@
       <c r="E13" s="58"/>
       <c r="F13" s="59">
         <f ca="1">TODAY()+5</f>
-        <v>46040</v>
+        <v>46075</v>
       </c>
       <c r="G13" s="60">
         <v>1</v>
@@ -18663,7 +18663,7 @@
         <v/>
       </c>
     </row>
-    <row r="14" spans="1:68" s="1" customFormat="1" ht="40.15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:68" s="1" customFormat="1" ht="40.15" customHeight="1">
       <c r="A14" s="9"/>
       <c r="B14" s="61" t="s">
         <v>12</v>
@@ -18677,7 +18677,7 @@
       </c>
       <c r="F14" s="59">
         <f ca="1">F12-3</f>
-        <v>46032</v>
+        <v>46067</v>
       </c>
       <c r="G14" s="60">
         <v>10</v>
@@ -18908,7 +18908,7 @@
         <v/>
       </c>
     </row>
-    <row r="15" spans="1:68" s="1" customFormat="1" ht="40.15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:68" s="1" customFormat="1" ht="40.15" customHeight="1">
       <c r="A15" s="9"/>
       <c r="B15" s="61" t="s">
         <v>13</v>
@@ -18920,7 +18920,7 @@
       <c r="E15" s="58"/>
       <c r="F15" s="59">
         <f ca="1">F12+20</f>
-        <v>46055</v>
+        <v>46090</v>
       </c>
       <c r="G15" s="60">
         <v>1</v>
@@ -19151,7 +19151,7 @@
         <v/>
       </c>
     </row>
-    <row r="16" spans="1:68" s="1" customFormat="1" ht="40.15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:68" s="1" customFormat="1" ht="40.15" customHeight="1">
       <c r="A16" s="9"/>
       <c r="B16" s="61" t="s">
         <v>14</v>
@@ -19165,7 +19165,7 @@
       </c>
       <c r="F16" s="59">
         <f ca="1">F12+6</f>
-        <v>46041</v>
+        <v>46076</v>
       </c>
       <c r="G16" s="60">
         <v>6</v>
@@ -19396,7 +19396,7 @@
         <v/>
       </c>
     </row>
-    <row r="17" spans="1:64" s="1" customFormat="1" ht="40.15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:64" s="1" customFormat="1" ht="40.15" customHeight="1">
       <c r="A17" s="10"/>
       <c r="B17" s="113" t="s">
         <v>15</v>
@@ -19632,7 +19632,7 @@
         <v/>
       </c>
     </row>
-    <row r="18" spans="1:64" s="1" customFormat="1" ht="40.15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:64" s="1" customFormat="1" ht="40.15" customHeight="1">
       <c r="A18" s="10"/>
       <c r="B18" s="61" t="s">
         <v>10</v>
@@ -19646,7 +19646,7 @@
       </c>
       <c r="F18" s="59">
         <f ca="1">F12+6</f>
-        <v>46041</v>
+        <v>46076</v>
       </c>
       <c r="G18" s="60">
         <v>13</v>
@@ -19877,7 +19877,7 @@
         <v/>
       </c>
     </row>
-    <row r="19" spans="1:64" s="1" customFormat="1" ht="40.15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:64" s="1" customFormat="1" ht="40.15" customHeight="1">
       <c r="A19" s="9"/>
       <c r="B19" s="61" t="s">
         <v>11</v>
@@ -19891,7 +19891,7 @@
       </c>
       <c r="F19" s="59">
         <f ca="1">F18+2</f>
-        <v>46043</v>
+        <v>46078</v>
       </c>
       <c r="G19" s="60">
         <v>9</v>
@@ -20122,7 +20122,7 @@
         <v/>
       </c>
     </row>
-    <row r="20" spans="1:64" s="1" customFormat="1" ht="40.15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:64" s="1" customFormat="1" ht="40.15" customHeight="1">
       <c r="A20" s="9"/>
       <c r="B20" s="61" t="s">
         <v>12</v>
@@ -20136,7 +20136,7 @@
       </c>
       <c r="F20" s="59">
         <f ca="1">F19+5</f>
-        <v>46048</v>
+        <v>46083</v>
       </c>
       <c r="G20" s="60">
         <v>11</v>
@@ -20367,7 +20367,7 @@
         <v/>
       </c>
     </row>
-    <row r="21" spans="1:64" s="1" customFormat="1" ht="40.15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:64" s="1" customFormat="1" ht="40.15" customHeight="1">
       <c r="A21" s="9"/>
       <c r="B21" s="61" t="s">
         <v>13</v>
@@ -20379,7 +20379,7 @@
       <c r="E21" s="58"/>
       <c r="F21" s="59">
         <f ca="1">F20+2</f>
-        <v>46050</v>
+        <v>46085</v>
       </c>
       <c r="G21" s="60">
         <v>1</v>
@@ -20610,7 +20610,7 @@
         <v/>
       </c>
     </row>
-    <row r="22" spans="1:64" s="1" customFormat="1" ht="40.15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:64" s="1" customFormat="1" ht="40.15" customHeight="1">
       <c r="A22" s="9"/>
       <c r="B22" s="61" t="s">
         <v>14</v>
@@ -20620,7 +20620,7 @@
       <c r="E22" s="58"/>
       <c r="F22" s="59">
         <f ca="1">F21+1</f>
-        <v>46051</v>
+        <v>46086</v>
       </c>
       <c r="G22" s="60">
         <v>24</v>
@@ -20851,7 +20851,7 @@
         <v/>
       </c>
     </row>
-    <row r="23" spans="1:64" s="1" customFormat="1" ht="40.15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:64" s="1" customFormat="1" ht="40.15" customHeight="1">
       <c r="A23" s="9"/>
       <c r="B23" s="113" t="s">
         <v>16</v>
@@ -21087,7 +21087,7 @@
         <v/>
       </c>
     </row>
-    <row r="24" spans="1:64" s="1" customFormat="1" ht="40.15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:64" s="1" customFormat="1" ht="40.15" customHeight="1">
       <c r="A24" s="9"/>
       <c r="B24" s="61" t="s">
         <v>10</v>
@@ -21099,7 +21099,7 @@
       <c r="E24" s="58"/>
       <c r="F24" s="59">
         <f ca="1">F12+15</f>
-        <v>46050</v>
+        <v>46085</v>
       </c>
       <c r="G24" s="60">
         <v>4</v>
@@ -21330,7 +21330,7 @@
         <v/>
       </c>
     </row>
-    <row r="25" spans="1:64" s="1" customFormat="1" ht="40.15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:64" s="1" customFormat="1" ht="40.15" customHeight="1">
       <c r="A25" s="9"/>
       <c r="B25" s="61" t="s">
         <v>11</v>
@@ -21342,7 +21342,7 @@
       <c r="E25" s="58"/>
       <c r="F25" s="59">
         <f ca="1">F24+3</f>
-        <v>46053</v>
+        <v>46088</v>
       </c>
       <c r="G25" s="60">
         <v>14</v>
@@ -21573,7 +21573,7 @@
         <v/>
       </c>
     </row>
-    <row r="26" spans="1:64" s="1" customFormat="1" ht="40.15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:64" s="1" customFormat="1" ht="40.15" customHeight="1">
       <c r="A26" s="9"/>
       <c r="B26" s="61" t="s">
         <v>12</v>
@@ -21585,7 +21585,7 @@
       <c r="E26" s="58"/>
       <c r="F26" s="59">
         <f ca="1">F25+15</f>
-        <v>46068</v>
+        <v>46103</v>
       </c>
       <c r="G26" s="60">
         <v>6</v>
@@ -21816,7 +21816,7 @@
         <v/>
       </c>
     </row>
-    <row r="27" spans="1:64" s="1" customFormat="1" ht="40.15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:64" s="1" customFormat="1" ht="40.15" customHeight="1">
       <c r="A27" s="9"/>
       <c r="B27" s="61" t="s">
         <v>13</v>
@@ -21828,7 +21828,7 @@
       <c r="E27" s="58"/>
       <c r="F27" s="59">
         <f ca="1">F21+22</f>
-        <v>46072</v>
+        <v>46107</v>
       </c>
       <c r="G27" s="60">
         <v>3</v>
@@ -22059,7 +22059,7 @@
         <v/>
       </c>
     </row>
-    <row r="28" spans="1:64" s="1" customFormat="1" ht="40.15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:64" s="1" customFormat="1" ht="40.15" customHeight="1">
       <c r="A28" s="9"/>
       <c r="B28" s="61" t="s">
         <v>14</v>
@@ -22071,7 +22071,7 @@
       <c r="E28" s="58"/>
       <c r="F28" s="59">
         <f ca="1">F16</f>
-        <v>46041</v>
+        <v>46076</v>
       </c>
       <c r="G28" s="60">
         <v>19</v>
@@ -22302,7 +22302,7 @@
         <v/>
       </c>
     </row>
-    <row r="29" spans="1:64" s="1" customFormat="1" ht="40.15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:64" s="1" customFormat="1" ht="40.15" customHeight="1">
       <c r="A29" s="9"/>
       <c r="B29" s="113" t="s">
         <v>17</v>
@@ -22538,7 +22538,7 @@
         <v/>
       </c>
     </row>
-    <row r="30" spans="1:64" s="1" customFormat="1" ht="40.15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:64" s="1" customFormat="1" ht="40.15" customHeight="1">
       <c r="A30" s="9"/>
       <c r="B30" s="61" t="s">
         <v>10</v>
@@ -22548,7 +22548,7 @@
       <c r="E30" s="58"/>
       <c r="F30" s="59">
         <f ca="1">F27+3</f>
-        <v>46075</v>
+        <v>46110</v>
       </c>
       <c r="G30" s="60">
         <v>15</v>
@@ -22779,7 +22779,7 @@
         <v/>
       </c>
     </row>
-    <row r="31" spans="1:64" s="1" customFormat="1" ht="40.15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:64" s="1" customFormat="1" ht="40.15" customHeight="1">
       <c r="A31" s="9"/>
       <c r="B31" s="61" t="s">
         <v>11</v>
@@ -22789,7 +22789,7 @@
       <c r="E31" s="58"/>
       <c r="F31" s="59">
         <f ca="1">F30+14</f>
-        <v>46089</v>
+        <v>46124</v>
       </c>
       <c r="G31" s="60">
         <v>5</v>
@@ -23020,7 +23020,7 @@
         <v/>
       </c>
     </row>
-    <row r="32" spans="1:64" s="1" customFormat="1" ht="40.15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:64" s="1" customFormat="1" ht="40.15" customHeight="1">
       <c r="A32" s="9"/>
       <c r="B32" s="61" t="s">
         <v>12</v>
@@ -23032,7 +23032,7 @@
       <c r="E32" s="58"/>
       <c r="F32" s="59">
         <f ca="1">F31+42</f>
-        <v>46131</v>
+        <v>46166</v>
       </c>
       <c r="G32" s="60">
         <v>1</v>
@@ -23263,7 +23263,7 @@
         <v/>
       </c>
     </row>
-    <row r="33" spans="1:65" s="1" customFormat="1" ht="40.15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:65" s="1" customFormat="1" ht="40.15" customHeight="1">
       <c r="A33" s="9"/>
       <c r="B33" s="61" t="s">
         <v>13</v>
@@ -23499,7 +23499,7 @@
         <v/>
       </c>
     </row>
-    <row r="34" spans="1:65" s="1" customFormat="1" ht="40.15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:65" s="1" customFormat="1" ht="40.15" customHeight="1">
       <c r="A34" s="9"/>
       <c r="B34" s="61" t="s">
         <v>14</v>
@@ -23735,7 +23735,7 @@
         <v/>
       </c>
     </row>
-    <row r="35" spans="1:65" s="1" customFormat="1" ht="40.15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:65" s="1" customFormat="1" ht="40.15" customHeight="1">
       <c r="A35" s="9"/>
       <c r="B35" s="61"/>
       <c r="C35" s="57"/>
@@ -23970,7 +23970,7 @@
       </c>
       <c r="BM35" s="86"/>
     </row>
-    <row r="36" spans="1:65" s="1" customFormat="1" ht="40.15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:65" s="1" customFormat="1" ht="40.15" customHeight="1">
       <c r="A36" s="10"/>
       <c r="B36" s="115" t="s">
         <v>18</v>
@@ -24038,12 +24038,12 @@
       <c r="BK36" s="84"/>
       <c r="BL36" s="84"/>
     </row>
-    <row r="37" spans="1:65" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:65" ht="30" customHeight="1">
       <c r="D37" s="4"/>
       <c r="G37" s="11"/>
       <c r="H37" s="3"/>
     </row>
-    <row r="38" spans="1:65" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:65" ht="30" customHeight="1">
       <c r="D38" s="5"/>
     </row>
   </sheetData>
@@ -24495,6 +24495,15 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <_ip_UnifiedCompliancePolicyUIAction xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
@@ -24512,15 +24521,6 @@
     <MediaServiceKeyPoints xmlns="71af3243-3dd4-4a8d-8c0d-dd76da1f02a5" xsi:nil="true"/>
   </documentManagement>
 </p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -24545,6 +24545,14 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{BAF2F40C-D12E-4644-AA6E-31E499F048DC}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6CD6AD73-D703-40CF-AB8D-72E6A3921BEB}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
@@ -24554,12 +24562,4 @@
     <ds:schemaRef ds:uri="230e9df3-be65-4c73-a93b-d1236ebd677e"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{BAF2F40C-D12E-4644-AA6E-31E499F048DC}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>